<commit_message>
PM log: March annuals confirmed at installation; AED1 model resolved
</commit_message>
<xml_diff>
--- a/life-safety/Life-Safety-PM-Log.xlsx
+++ b/life-safety/Life-Safety-PM-Log.xlsx
@@ -1944,8 +1944,10 @@
         <v>11</v>
       </c>
       <c r="E29" s="6"/>
-      <c r="F29" s="7" t="s">
-        <v>37</v>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1962,8 +1964,10 @@
         <v>11</v>
       </c>
       <c r="E30" s="6"/>
-      <c r="F30" s="7" t="s">
-        <v>37</v>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1980,8 +1984,10 @@
         <v>11</v>
       </c>
       <c r="E31" s="6"/>
-      <c r="F31" s="7" t="s">
-        <v>37</v>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1998,8 +2004,10 @@
         <v>11</v>
       </c>
       <c r="E32" s="6"/>
-      <c r="F32" s="7" t="s">
-        <v>37</v>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2016,8 +2024,10 @@
         <v>11</v>
       </c>
       <c r="E33" s="6"/>
-      <c r="F33" s="7" t="s">
-        <v>37</v>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2034,8 +2044,10 @@
         <v>11</v>
       </c>
       <c r="E34" s="6"/>
-      <c r="F34" s="7" t="s">
-        <v>37</v>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2052,8 +2064,10 @@
         <v>11</v>
       </c>
       <c r="E35" s="6"/>
-      <c r="F35" s="7" t="s">
-        <v>37</v>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2070,8 +2084,10 @@
         <v>11</v>
       </c>
       <c r="E36" s="6"/>
-      <c r="F36" s="7" t="s">
-        <v>37</v>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2128,8 +2144,10 @@
         <v>11</v>
       </c>
       <c r="E39" s="6"/>
-      <c r="F39" s="7" t="s">
-        <v>37</v>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2326,8 +2344,10 @@
         <v>11</v>
       </c>
       <c r="E49" s="6"/>
-      <c r="F49" s="7" t="s">
-        <v>37</v>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annual service confirmed done at installation, March 2026.</t>
+        </is>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7777,8 +7797,10 @@
         <f aca="false">IF($L6="","NOT LOGGED",IF($L6&lt;=0,"OVERDUE",IF($L6&lt;=IF(MIN($F6,$H6,$J6)=$F6,Intervals!$C$26,Intervals!$C$38),"DUE SOON","OK")))</f>
         <v>OK</v>
       </c>
-      <c r="N6" s="39" t="s">
-        <v>244</v>
+      <c r="N6" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PlusTrac record X25G370264, "Shipping Office Area", licensed PlusRx (license expires 02/18/2027), monthly interval. Model confirmed as ZOLL AED 3 (resolved 10/29/2026). Battery pack SN AU24LAD3904, label INSTALL BY 12/20/2026.</t>
+        </is>
       </c>
       <c r="O6" s="27" t="str">
         <f aca="false">IF($E6="","",IF(SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A6)*('Inspection History'!$C$6:$C$20000="Readiness Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$E6)*ROW('Inspection History'!$A$6:$A$20000)))=0,"",INDEX('Inspection History'!$E:$E,SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A6)*('Inspection History'!$C$6:$C$20000="Readiness Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$E6)*ROW('Inspection History'!$A$6:$A$20000))))&amp;""))</f>

</xml_diff>

<commit_message>
PM log: EW2 replaced and relocated; AED2 tracked in PlusTrac
</commit_message>
<xml_diff>
--- a/life-safety/Life-Safety-PM-Log.xlsx
+++ b/life-safety/Life-Safety-PM-Log.xlsx
@@ -7343,8 +7343,10 @@
       <c r="A7" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="29" t="s">
-        <v>221</v>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One column (about 20 ft) from the hi-lo battery chargers</t>
+        </is>
       </c>
       <c r="C7" s="24" t="s">
         <v>120</v>
@@ -7385,8 +7387,10 @@
         <f aca="false">IF($K7="","NOT LOGGED",IF($K7&lt;=0,"OVERDUE",IF($K7&lt;=Intervals!$C$27,"DUE SOON","OK")))</f>
         <v>OK</v>
       </c>
-      <c r="M7" s="24" t="s">
-        <v>222</v>
+      <c r="M7" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Larger self-contained eyewash, mounted one column (about 20 ft) from the hi-lo battery chargers. It replaces the Gravit-Eye unit installed 10/19/2026, which itself replaced the squeeze bottles.</t>
+        </is>
       </c>
       <c r="N7" s="27" t="str">
         <f aca="false">IF($D7="","",IF(SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A7)*('Inspection History'!$C$6:$C$20000="Weekly Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$D7)*ROW('Inspection History'!$A$6:$A$20000)))=0,"",INDEX('Inspection History'!$E:$E,SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A7)*('Inspection History'!$C$6:$C$20000="Weekly Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$D7)*ROW('Inspection History'!$A$6:$A$20000))))&amp;""))</f>
@@ -7854,8 +7858,10 @@
         <f aca="false">IF($L7="","NOT LOGGED",IF($L7&lt;=0,"OVERDUE",IF($L7&lt;=IF(MIN($F7,$H7,$J7)=$F7,Intervals!$C$26,Intervals!$C$38),"DUE SOON","OK")))</f>
         <v>OK</v>
       </c>
-      <c r="N7" s="39" t="s">
-        <v>247</v>
+      <c r="N7" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PlusTrac record AX25G370194, "Supervisor's Office Area", ZOLL AED 3, monthly interval. Tracked in PlusTrac and showing Compliant as of 10/29/2026 (last PlusTrac inspection 09/30/2026). Battery pack SN AU24LAD3856, label INSTALL BY 12/20/2026.</t>
+        </is>
       </c>
       <c r="O7" s="27" t="str">
         <f aca="false">IF($E7="","",IF(SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A7)*('Inspection History'!$C$6:$C$20000="Readiness Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$E7)*ROW('Inspection History'!$A$6:$A$20000)))=0,"",INDEX('Inspection History'!$E:$E,SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A7)*('Inspection History'!$C$6:$C$20000="Readiness Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$E7)*ROW('Inspection History'!$A$6:$A$20000))))&amp;""))</f>

</xml_diff>

<commit_message>
PM log: EW2 location relative to relocated hi-lo chargers
</commit_message>
<xml_diff>
--- a/life-safety/Life-Safety-PM-Log.xlsx
+++ b/life-safety/Life-Safety-PM-Log.xlsx
@@ -7345,7 +7345,7 @@
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">One column (about 20 ft) from the hi-lo battery chargers</t>
+          <t xml:space="preserve">One column (about 20 ft) from the hi-lo battery chargers, which sit on the column between the 610 and 720 Ton</t>
         </is>
       </c>
       <c r="C7" s="24" t="s">
@@ -7389,7 +7389,7 @@
       </c>
       <c r="M7" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Larger self-contained eyewash, mounted one column (about 20 ft) from the hi-lo battery chargers. It replaces the Gravit-Eye unit installed 10/19/2026, which itself replaced the squeeze bottles.</t>
+          <t xml:space="preserve">Larger self-contained eyewash, filled on site, delivers the full 15-minute flush required by ANSI Z358.1. Mounted one column (about 20 ft) from the hi-lo battery chargers. It replaces the Gravit-Eye unit installed 10/19/2026, which itself replaced the squeeze bottles.</t>
         </is>
       </c>
       <c r="N7" s="27" t="str">

</xml_diff>

<commit_message>
PM log: EW5 installed and inspected by J. Godek 10/19 (first service date)
</commit_message>
<xml_diff>
--- a/life-safety/Life-Safety-PM-Log.xlsx
+++ b/life-safety/Life-Safety-PM-Log.xlsx
@@ -3407,9 +3407,15 @@
       <c r="D108" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E108" s="6"/>
-      <c r="F108" s="7" t="s">
-        <v>73</v>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">J. Godek</t>
+        </is>
+      </c>
+      <c r="F108" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Installed and inspected by J. Godek; first service date.</t>
+        </is>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3425,9 +3431,15 @@
       <c r="D109" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E109" s="6"/>
-      <c r="F109" s="7" t="s">
-        <v>73</v>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">J. Godek</t>
+        </is>
+      </c>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Installed and filled by J. Godek; first service date.</t>
+        </is>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3443,9 +3455,15 @@
       <c r="D110" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E110" s="6"/>
-      <c r="F110" s="7" t="s">
-        <v>73</v>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">J. Godek</t>
+        </is>
+      </c>
+      <c r="F110" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Installed and activated by J. Godek; first service date.</t>
+        </is>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7547,8 +7565,10 @@
         <f aca="false">IF($K10="","NOT LOGGED",IF($K10&lt;=0,"OVERDUE",IF($K10&lt;=Intervals!$C$27,"DUE SOON","OK")))</f>
         <v>OK</v>
       </c>
-      <c r="M10" s="24" t="s">
-        <v>225</v>
+      <c r="M10" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guardian gravity-fed self-contained eyewash on the column behind the 1400 Ton, beside the spill kit and oily-waste can. Installed and inspected by J. Godek on 10/19/2026, which is its first service date for the weekly activation, annual inspection and fluid change.</t>
+        </is>
       </c>
       <c r="N10" s="27" t="str">
         <f aca="false">IF($D10="","",IF(SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A10)*('Inspection History'!$C$6:$C$20000="Weekly Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$D10)*ROW('Inspection History'!$A$6:$A$20000)))=0,"",INDEX('Inspection History'!$E:$E,SUMPRODUCT(MAX(('Inspection History'!$B$6:$B$20000=$A10)*('Inspection History'!$C$6:$C$20000="Weekly Check")*('Inspection History'!$D$6:$D$20000="Pass")*('Inspection History'!$A$6:$A$20000=$D10)*ROW('Inspection History'!$A$6:$A$20000))))&amp;""))</f>

</xml_diff>

<commit_message>
Scan-to-log: label codes unlock Pass/Fail, timestamps, no bulk pass; history tab protected
</commit_message>
<xml_diff>
--- a/life-safety/Life-Safety-PM-Log.xlsx
+++ b/life-safety/Life-Safety-PM-Log.xlsx
@@ -1455,7 +1455,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -1464,6 +1464,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1476,9 +1477,11 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
+    <row r="2" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One row per inspection, never overwritten. Routine checks are logged by scanning each device's QR label; vendor and annual work is added here by hand (Review &gt; Unprotect Sheet first, then protect it again). Every tab's Last date, Next date and status update from this tab. Only Pass rows count toward the schedule: a Fail stays on the record but does not reset the clock. Logged at shows the clock time and method of scanned entries.</t>
+        </is>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1515,6 +1518,11 @@
       <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Logged at</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="n">
@@ -4025,6 +4033,7 @@
       <c r="F141" s="7"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" objects="true" scenarios="true" formatColumns="false" formatRows="false" sort="false" autoFilter="false"/>
   <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>

</xml_diff>